<commit_message>
feature: alinear lógica anual y filtros de gastos con main
Se unifica el cálculo de masa salarial/cobertura anual (incluyendo hardcode histórico y 2025-2026 dinámico), y se corrigen ajustes de UI/UX en mensual, anual y gastos para igualar comportamiento y visual de main.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/backend/inputs/reca.xlsx
+++ b/backend/inputs/reca.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10404"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10426"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ivanrodriguez/Documents/Antigravity/Coparticipacion/main/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5A764CB-0969-6642-8375-0572DA46BAC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64F849AD-533A-FE43-89FC-C77A6896CC8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="19200" windowHeight="21000" xr2:uid="{E327F0F6-7896-FA43-9329-53B85594D54E}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="17280" windowHeight="21680" xr2:uid="{E327F0F6-7896-FA43-9329-53B85594D54E}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -1269,6 +1269,35 @@
         <v>0</v>
       </c>
     </row>
+    <row r="29" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A29">
+        <v>2026</v>
+      </c>
+      <c r="B29">
+        <v>4</v>
+      </c>
+      <c r="C29" s="1">
+        <v>5275915851.8100004</v>
+      </c>
+      <c r="D29" s="1">
+        <v>537540232.57000005</v>
+      </c>
+      <c r="E29" s="1">
+        <v>60012511.950000003</v>
+      </c>
+      <c r="F29" s="1">
+        <v>5472368435.7299995</v>
+      </c>
+      <c r="G29" s="1">
+        <v>73033897.890000001</v>
+      </c>
+      <c r="H29" s="1">
+        <v>32059956612.02</v>
+      </c>
+      <c r="I29" s="1">
+        <v>0</v>
+      </c>
+    </row>
     <row r="30" spans="1:17" x14ac:dyDescent="0.2">
       <c r="F30" s="1"/>
       <c r="G30" s="1"/>

</xml_diff>